<commit_message>
feat: support production API_BASE and HTTPS protocol in automation runners
</commit_message>
<xml_diff>
--- a/tests/test_results.xlsx
+++ b/tests/test_results.xlsx
@@ -579,11 +579,11 @@
         <v>200</v>
       </c>
       <c r="L2" t="n">
-        <v>118</v>
+        <v>163</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"token": "eyJhbGciOiJIUzI1NiIsInR5cCI6IkpXVCJ9.eyJpZCI6ImNtcnN5cmk1YjAwMDBsY2I0Z2hzd2I4ZTUiLCJ1c2VybmFtZSI6ImFkbWluIiwicm9sZSI6IlNVUEVSQURNSU4iLCJpYXQiOjE3ODQ3MDI0MjIsImV4cC</t>
+          <t>{"success": true, "data": {"token": "eyJhbGciOiJIUzI1NiIsInR5cCI6IkpXVCJ9.eyJpZCI6ImNtcnN5cmk1YjAwMDBsY2I0Z2hzd2I4ZTUiLCJ1c2VybmFtZSI6ImFkbWluIiwicm9sZSI6IlNVUEVSQURNSU4iLCJpYXQiOjE3ODQ3MDMxMTcsImV4cC</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
         <v>401</v>
       </c>
       <c r="L3" t="n">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -697,7 +697,7 @@
         <v>200</v>
       </c>
       <c r="L4" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -754,7 +754,7 @@
         <v>200</v>
       </c>
       <c r="L5" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
         <v>200</v>
       </c>
       <c r="L6" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -872,11 +872,11 @@
         <v>201</v>
       </c>
       <c r="L7" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"id": "cmrvpqqtg002dlcsgf9xeymmm", "eventId": "cmrvgy4ej0000lcg4jjl9dux1", "name": "Excel Gate Door 1", "location": "Hall 1", "isActive": true, "sortOrder": 10, "createdAt":</t>
+          <t>{"success": true, "data": {"id": "cmrvq5mwi002wlcsgjrf5f2io", "eventId": "cmrvgy4ej0000lcg4jjl9dux1", "name": "Excel Gate Door 1", "location": "Hall 1", "isActive": true, "sortOrder": 10, "createdAt":</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>{"eventId": "cmrvgy4ej0000lcg4jjl9dux1", "fullName": "Excel Tester Guest", "email": "excel.test.1784702422863@example.com", "phone": "0899999999", "company": "Excel QA Corp"}</t>
+          <t>{"eventId": "cmrvgy4ej0000lcg4jjl9dux1", "fullName": "Excel Tester Guest", "email": "excel.test.1784703117635@example.com", "phone": "0899999999", "company": "Excel QA Corp"}</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -933,11 +933,11 @@
         <v>201</v>
       </c>
       <c r="L8" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"id": "cmrvpqqu8002glcsgnhupmmi0", "eventId": "cmrvgy4ej0000lcg4jjl9dux1", "fullName": "Excel Tester Guest", "email": "excel.test.1784702422863@example.com", "phone": "08999</t>
+          <t>{"success": true, "data": {"id": "cmrvq5mxk002zlcsgxmff7f50", "eventId": "cmrvgy4ej0000lcg4jjl9dux1", "fullName": "Excel Tester Guest", "email": "excel.test.1784703117635@example.com", "phone": "08999</t>
         </is>
       </c>
     </row>
@@ -969,7 +969,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>{"registrationId": "cmrvpqqu8002glcsgnhupmmi0", "checkinPointId": "cmrvpqqtg002dlcsgf9xeymmm", "method": "MANUAL"}</t>
+          <t>{"registrationId": "cmrvq5mxk002zlcsgxmff7f50", "checkinPointId": "cmrvq5mwi002wlcsgjrf5f2io", "method": "MANUAL"}</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -994,11 +994,11 @@
         <v>201</v>
       </c>
       <c r="L9" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"checkin": {"id": "cmrvpqquw002jlcsgdmarwb6d", "registrationId": "cmrvpqqu8002glcsgnhupmmi0", "checkinPointId": "cmrvpqqtg002dlcsgf9xeymmm", "checkinTime": "2026-07-22T06:40</t>
+          <t>{"success": true, "data": {"checkin": {"id": "cmrvq5myj0032lcsg68wwjoe8", "registrationId": "cmrvq5mxk002zlcsgxmff7f50", "checkinPointId": "cmrvq5mwi002wlcsgjrf5f2io", "checkinTime": "2026-07-22T06:51</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
         <v>200</v>
       </c>
       <c r="L10" t="n">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1112,11 +1112,11 @@
         <v>201</v>
       </c>
       <c r="L11" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"id": "cmrvpqqvx002mlcsgtvnoje3u", "eventId": "cmrvgy4ej0000lcg4jjl9dux1", "prizeId": "cmrvgy4fj000alcg4qurjil4y", "status": "PENDING", "drawCount": 1, "startedAt": null, "e</t>
+          <t>{"success": true, "data": {"id": "cmrvq5n0p0035lcsgnmglun7w", "eventId": "cmrvgy4ej0000lcg4jjl9dux1", "prizeId": "cmrvgy4fj000alcg4qurjil4y", "status": "PENDING", "drawCount": 1, "startedAt": null, "e</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1143,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>/api/draws/cmrvpqqvx002mlcsgtvnoje3u/spin</t>
+          <t>/api/draws/cmrvq5n0p0035lcsgnmglun7w/spin</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1173,11 +1173,11 @@
         <v>200</v>
       </c>
       <c r="L12" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"winners": [{"id": "cmrvmonyq000mlcsg5pd907ed", "fullName": "Automation Test Guest", "department": "Software Testing", "company": "Antigravity QA Labs", "employeeType": null</t>
+          <t>{"success": true, "data": {"winners": [{"id": "cmrvq5mxk002zlcsgxmff7f50", "fullName": "Excel Tester Guest", "department": null, "company": "Excel QA Corp", "employeeType": null}], "candidates": 36}}</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>/api/draws/winners/cmrvpqqx1002plcsg6vok78t3</t>
+          <t>/api/draws/winners/cmrvq5n2a0038lcsgnafwcxsn</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1234,11 +1234,11 @@
         <v>200</v>
       </c>
       <c r="L13" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"id": "cmrvpqqx1002plcsg6vok78t3", "drawSessionId": "cmrvpqqvx002mlcsgtvnoje3u", "registrationId": "cmrvmonyq000mlcsg5pd907ed", "prizeId": "cmrvgy4fj000alcg4qurjil4y", "stat</t>
+          <t>{"success": true, "data": {"id": "cmrvq5n2a0038lcsgnafwcxsn", "drawSessionId": "cmrvq5n0p0035lcsgnmglun7w", "registrationId": "cmrvq5mxk002zlcsgxmff7f50", "prizeId": "cmrvgy4fj000alcg4qurjil4y", "stat</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>/api/draws/winners/cmrvpqqx1002plcsg6vok78t3</t>
+          <t>/api/draws/winners/cmrvq5n2a0038lcsgnafwcxsn</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -1291,7 +1291,7 @@
         <v>200</v>
       </c>
       <c r="L14" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: add native prod / test CLI arguments support for automation test commands
</commit_message>
<xml_diff>
--- a/tests/test_results.xlsx
+++ b/tests/test_results.xlsx
@@ -579,11 +579,11 @@
         <v>200</v>
       </c>
       <c r="L2" t="n">
-        <v>163</v>
+        <v>122</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"token": "eyJhbGciOiJIUzI1NiIsInR5cCI6IkpXVCJ9.eyJpZCI6ImNtcnN5cmk1YjAwMDBsY2I0Z2hzd2I4ZTUiLCJ1c2VybmFtZSI6ImFkbWluIiwicm9sZSI6IlNVUEVSQURNSU4iLCJpYXQiOjE3ODQ3MDMxMTcsImV4cC</t>
+          <t>{"success": true, "data": {"token": "eyJhbGciOiJIUzI1NiIsInR5cCI6IkpXVCJ9.eyJpZCI6ImNtcnN5cmk1YjAwMDBsY2I0Z2hzd2I4ZTUiLCJ1c2VybmFtZSI6ImFkbWluIiwicm9sZSI6IlNVUEVSQURNSU4iLCJpYXQiOjE3ODQ3MDM3OTQsImV4cC</t>
         </is>
       </c>
     </row>
@@ -697,11 +697,11 @@
         <v>200</v>
       </c>
       <c r="L4" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>{"success": true, "data": [{"id": "cmrvgy4ej0000lcg4jjl9dux1", "name": "Tech Conference 2026", "description": "Annual technology conference with workshops, talks, and networking", "venue": "Bangkok Co</t>
+          <t>{"success": true, "data": [{"id": "cmrvqjvqm0000lcswueuniggq", "name": "Tech Conference 2026", "description": "Annual technology conference with workshops, talks, and networking", "venue": "Bangkok Co</t>
         </is>
       </c>
     </row>
@@ -728,7 +728,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>/api/events/cmrvgy4ej0000lcg4jjl9dux1</t>
+          <t>/api/events/cmrvqjvqm0000lcswueuniggq</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -754,11 +754,11 @@
         <v>200</v>
       </c>
       <c r="L5" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"id": "cmrvgy4ej0000lcg4jjl9dux1", "name": "Tech Conference 2026", "description": "Annual technology conference with workshops, talks, and networking", "venue": "Bangkok Con</t>
+          <t>{"success": true, "data": {"id": "cmrvqjvqm0000lcswueuniggq", "name": "Tech Conference 2026", "description": "Annual technology conference with workshops, talks, and networking", "venue": "Bangkok Con</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>/api/checkin/points?eventId=cmrvgy4ej0000lcg4jjl9dux1</t>
+          <t>/api/checkin/points?eventId=cmrvqjvqm0000lcswueuniggq</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -811,11 +811,11 @@
         <v>200</v>
       </c>
       <c r="L6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>{"success": true, "data": [{"id": "cmrvgy4eq0002lcg4dhxbk1yn", "eventId": "cmrvgy4ej0000lcg4jjl9dux1", "name": "Main Entrance", "location": "Hall A - Ground Floor", "isActive": true, "sortOrder": 1, "</t>
+          <t>{"success": true, "data": [{"id": "cmrvqjvqu0002lcswyyqtzxlt", "eventId": "cmrvqjvqm0000lcswueuniggq", "name": "Main Entrance", "location": "Hall A - Ground Floor", "isActive": true, "sortOrder": 1, "</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>{"eventId": "cmrvgy4ej0000lcg4jjl9dux1", "name": "Excel Gate Door 1", "location": "Hall 1", "isActive": true, "sortOrder": 10}</t>
+          <t>{"eventId": "cmrvqjvqm0000lcswueuniggq", "name": "Excel Gate Door 1", "location": "Hall 1", "isActive": true, "sortOrder": 10}</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -872,11 +872,11 @@
         <v>201</v>
       </c>
       <c r="L7" t="n">
-        <v>19</v>
+        <v>58</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"id": "cmrvq5mwi002wlcsgjrf5f2io", "eventId": "cmrvgy4ej0000lcg4jjl9dux1", "name": "Excel Gate Door 1", "location": "Hall 1", "isActive": true, "sortOrder": 10, "createdAt":</t>
+          <t>{"success": true, "data": {"id": "cmrvqk5le003xlcsgrrbkgwz6", "eventId": "cmrvqjvqm0000lcswueuniggq", "name": "Excel Gate Door 1", "location": "Hall 1", "isActive": true, "sortOrder": 10, "createdAt":</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>{"eventId": "cmrvgy4ej0000lcg4jjl9dux1", "fullName": "Excel Tester Guest", "email": "excel.test.1784703117635@example.com", "phone": "0899999999", "company": "Excel QA Corp"}</t>
+          <t>{"eventId": "cmrvqjvqm0000lcswueuniggq", "fullName": "Excel Tester Guest", "email": "excel.test.1784703795082@example.com", "phone": "0899999999", "company": "Excel QA Corp"}</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -933,11 +933,11 @@
         <v>201</v>
       </c>
       <c r="L8" t="n">
-        <v>40</v>
+        <v>66</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"id": "cmrvq5mxk002zlcsgxmff7f50", "eventId": "cmrvgy4ej0000lcg4jjl9dux1", "fullName": "Excel Tester Guest", "email": "excel.test.1784703117635@example.com", "phone": "08999</t>
+          <t>{"success": true, "data": {"id": "cmrvqk5nl0040lcsgl5jz45qp", "eventId": "cmrvqjvqm0000lcswueuniggq", "fullName": "Excel Tester Guest", "email": "excel.test.1784703795082@example.com", "phone": "08999</t>
         </is>
       </c>
     </row>
@@ -969,7 +969,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>{"registrationId": "cmrvq5mxk002zlcsgxmff7f50", "checkinPointId": "cmrvq5mwi002wlcsgjrf5f2io", "method": "MANUAL"}</t>
+          <t>{"registrationId": "cmrvqk5nl0040lcsgl5jz45qp", "checkinPointId": "cmrvqk5le003xlcsgrrbkgwz6", "method": "MANUAL"}</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -994,11 +994,11 @@
         <v>201</v>
       </c>
       <c r="L9" t="n">
-        <v>36</v>
+        <v>121</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"checkin": {"id": "cmrvq5myj0032lcsg68wwjoe8", "registrationId": "cmrvq5mxk002zlcsgxmff7f50", "checkinPointId": "cmrvq5mwi002wlcsgjrf5f2io", "checkinTime": "2026-07-22T06:51</t>
+          <t>{"success": true, "data": {"checkin": {"id": "cmrvqk5q20043lcsg0mi1ao5o", "registrationId": "cmrvqk5nl0040lcsgl5jz45qp", "checkinPointId": "cmrvqk5le003xlcsgrrbkgwz6", "checkinTime": "2026-07-22T07:03</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>/api/prizes?eventId=cmrvgy4ej0000lcg4jjl9dux1</t>
+          <t>/api/prizes?eventId=cmrvqjvqm0000lcswueuniggq</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -1051,11 +1051,11 @@
         <v>200</v>
       </c>
       <c r="L10" t="n">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>{"success": true, "data": [{"id": "cmrvgy4fj000clcg4p4ok73xt", "eventId": "cmrvgy4ej0000lcg4jjl9dux1", "name": "MacBook Pro 16\"", "description": "Apple MacBook Pro 16-inch M4 Pro", "image": null, "qu</t>
+          <t>{"success": true, "data": [{"id": "cmrvqjvrn000alcsw216ijgbl", "eventId": "cmrvqjvqm0000lcswueuniggq", "name": "MacBook Pro 16\"", "description": "Apple MacBook Pro 16-inch M4 Pro", "image": null, "qu</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1087,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>{"eventId": "cmrvgy4ej0000lcg4jjl9dux1", "prizeId": "cmrvgy4fj000alcg4qurjil4y", "drawCount": 1}</t>
+          <t>{"eventId": "cmrvqjvqm0000lcswueuniggq", "prizeId": "cmrvqjvrn000alcsw216ijgbl", "drawCount": 1}</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1112,11 +1112,11 @@
         <v>201</v>
       </c>
       <c r="L11" t="n">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"id": "cmrvq5n0p0035lcsgnmglun7w", "eventId": "cmrvgy4ej0000lcg4jjl9dux1", "prizeId": "cmrvgy4fj000alcg4qurjil4y", "status": "PENDING", "drawCount": 1, "startedAt": null, "e</t>
+          <t>{"success": true, "data": {"id": "cmrvqk5t90046lcsgtf7uoplm", "eventId": "cmrvqjvqm0000lcswueuniggq", "prizeId": "cmrvqjvrn000alcsw216ijgbl", "status": "PENDING", "drawCount": 1, "startedAt": null, "e</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1143,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>/api/draws/cmrvq5n0p0035lcsgnmglun7w/spin</t>
+          <t>/api/draws/cmrvqk5t90046lcsgtf7uoplm/spin</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1173,11 +1173,11 @@
         <v>200</v>
       </c>
       <c r="L12" t="n">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"winners": [{"id": "cmrvq5mxk002zlcsgxmff7f50", "fullName": "Excel Tester Guest", "department": null, "company": "Excel QA Corp", "employeeType": null}], "candidates": 36}}</t>
+          <t>{"success": true, "data": {"winners": [{"id": "cmrvqjvx70020lcsw64qrgb8g", "fullName": "Attendee 029", "department": "Finance", "company": "Tech Corp", "employeeType": "Contract"}], "candidates": 31}}</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>/api/draws/winners/cmrvq5n2a0038lcsgnafwcxsn</t>
+          <t>/api/draws/winners/cmrvqk5vb0049lcsg5y5vtfki</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1234,11 +1234,11 @@
         <v>200</v>
       </c>
       <c r="L13" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"id": "cmrvq5n2a0038lcsgnafwcxsn", "drawSessionId": "cmrvq5n0p0035lcsgnmglun7w", "registrationId": "cmrvq5mxk002zlcsgxmff7f50", "prizeId": "cmrvgy4fj000alcg4qurjil4y", "stat</t>
+          <t>{"success": true, "data": {"id": "cmrvqk5vb0049lcsg5y5vtfki", "drawSessionId": "cmrvqk5t90046lcsgtf7uoplm", "registrationId": "cmrvqjvx70020lcsw64qrgb8g", "prizeId": "cmrvqjvrn000alcsw216ijgbl", "stat</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>/api/draws/winners/cmrvq5n2a0038lcsgnafwcxsn</t>
+          <t>/api/draws/winners/cmrvqk5vb0049lcsg5y5vtfki</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: support dynamic custom Excel input and output file names
</commit_message>
<xml_diff>
--- a/tests/test_results.xlsx
+++ b/tests/test_results.xlsx
@@ -442,7 +442,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -579,11 +579,11 @@
         <v>200</v>
       </c>
       <c r="L2" t="n">
-        <v>122</v>
+        <v>166</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"token": "eyJhbGciOiJIUzI1NiIsInR5cCI6IkpXVCJ9.eyJpZCI6ImNtcnN5cmk1YjAwMDBsY2I0Z2hzd2I4ZTUiLCJ1c2VybmFtZSI6ImFkbWluIiwicm9sZSI6IlNVUEVSQURNSU4iLCJpYXQiOjE3ODQ3MDM3OTQsImV4cC</t>
+          <t>{"success": true, "data": {"token": "eyJhbGciOiJIUzI1NiIsInR5cCI6IkpXVCJ9.eyJpZCI6ImNtcnN5cmk1YjAwMDBsY2I0Z2hzd2I4ZTUiLCJ1c2VybmFtZSI6ImFkbWluIiwicm9sZSI6IlNVUEVSQURNSU4iLCJpYXQiOjE3ODQ3MDQxODEsImV4cC</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
         <v>401</v>
       </c>
       <c r="L3" t="n">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -754,7 +754,7 @@
         <v>200</v>
       </c>
       <c r="L5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
         <v>200</v>
       </c>
       <c r="L6" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -872,11 +872,11 @@
         <v>201</v>
       </c>
       <c r="L7" t="n">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"id": "cmrvqk5le003xlcsgrrbkgwz6", "eventId": "cmrvqjvqm0000lcswueuniggq", "name": "Excel Gate Door 1", "location": "Hall 1", "isActive": true, "sortOrder": 10, "createdAt":</t>
+          <t>{"success": true, "data": {"id": "cmrvqsfs3004glcsgywtg0rrx", "eventId": "cmrvqjvqm0000lcswueuniggq", "name": "Excel Gate Door 1", "location": "Hall 1", "isActive": true, "sortOrder": 10, "createdAt":</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>{"eventId": "cmrvqjvqm0000lcswueuniggq", "fullName": "Excel Tester Guest", "email": "excel.test.1784703795082@example.com", "phone": "0899999999", "company": "Excel QA Corp"}</t>
+          <t>{"eventId": "cmrvqjvqm0000lcswueuniggq", "fullName": "Excel Tester Guest", "email": "excel.test.1784704181489@example.com", "phone": "0899999999", "company": "Excel QA Corp"}</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -933,11 +933,11 @@
         <v>201</v>
       </c>
       <c r="L8" t="n">
-        <v>66</v>
+        <v>36</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"id": "cmrvqk5nl0040lcsgl5jz45qp", "eventId": "cmrvqjvqm0000lcswueuniggq", "fullName": "Excel Tester Guest", "email": "excel.test.1784703795082@example.com", "phone": "08999</t>
+          <t>{"success": true, "data": {"id": "cmrvqsft0004jlcsgg3gxvdc3", "eventId": "cmrvqjvqm0000lcswueuniggq", "fullName": "Excel Tester Guest", "email": "excel.test.1784704181489@example.com", "phone": "08999</t>
         </is>
       </c>
     </row>
@@ -969,7 +969,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>{"registrationId": "cmrvqk5nl0040lcsgl5jz45qp", "checkinPointId": "cmrvqk5le003xlcsgrrbkgwz6", "method": "MANUAL"}</t>
+          <t>{"registrationId": "cmrvqsft0004jlcsgg3gxvdc3", "checkinPointId": "cmrvqsfs3004glcsgywtg0rrx", "method": "MANUAL"}</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -994,11 +994,11 @@
         <v>201</v>
       </c>
       <c r="L9" t="n">
-        <v>121</v>
+        <v>34</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"checkin": {"id": "cmrvqk5q20043lcsg0mi1ao5o", "registrationId": "cmrvqk5nl0040lcsgl5jz45qp", "checkinPointId": "cmrvqk5le003xlcsgrrbkgwz6", "checkinTime": "2026-07-22T07:03</t>
+          <t>{"success": true, "data": {"checkin": {"id": "cmrvqsftw004mlcsgkf85b5ll", "registrationId": "cmrvqsft0004jlcsgg3gxvdc3", "checkinPointId": "cmrvqsfs3004glcsgywtg0rrx", "checkinTime": "2026-07-22T07:09</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
         <v>200</v>
       </c>
       <c r="L10" t="n">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1112,11 +1112,11 @@
         <v>201</v>
       </c>
       <c r="L11" t="n">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"id": "cmrvqk5t90046lcsgtf7uoplm", "eventId": "cmrvqjvqm0000lcswueuniggq", "prizeId": "cmrvqjvrn000alcsw216ijgbl", "status": "PENDING", "drawCount": 1, "startedAt": null, "e</t>
+          <t>{"success": true, "data": {"id": "cmrvqsfvu004plcsg88a1qlwd", "eventId": "cmrvqjvqm0000lcswueuniggq", "prizeId": "cmrvqjvrn000alcsw216ijgbl", "status": "PENDING", "drawCount": 1, "startedAt": null, "e</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1143,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>/api/draws/cmrvqk5t90046lcsgtf7uoplm/spin</t>
+          <t>/api/draws/cmrvqsfvu004plcsg88a1qlwd/spin</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1173,11 +1173,11 @@
         <v>200</v>
       </c>
       <c r="L12" t="n">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"winners": [{"id": "cmrvqjvx70020lcsw64qrgb8g", "fullName": "Attendee 029", "department": "Finance", "company": "Tech Corp", "employeeType": "Contract"}], "candidates": 31}}</t>
+          <t>{"success": true, "data": {"winners": [{"id": "cmrvqjvws001ulcsw31id462s", "fullName": "Attendee 026", "department": "Engineering", "company": "Tech Corp", "employeeType": "Intern"}], "candidates": 32</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>/api/draws/winners/cmrvqk5vb0049lcsg5y5vtfki</t>
+          <t>/api/draws/winners/cmrvqsfx6004slcsg3uve7y2u</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1234,11 +1234,11 @@
         <v>200</v>
       </c>
       <c r="L13" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>{"success": true, "data": {"id": "cmrvqk5vb0049lcsg5y5vtfki", "drawSessionId": "cmrvqk5t90046lcsgtf7uoplm", "registrationId": "cmrvqjvx70020lcsw64qrgb8g", "prizeId": "cmrvqjvrn000alcsw216ijgbl", "stat</t>
+          <t>{"success": true, "data": {"id": "cmrvqsfx6004slcsg3uve7y2u", "drawSessionId": "cmrvqsfvu004plcsg88a1qlwd", "registrationId": "cmrvqjvws001ulcsw31id462s", "prizeId": "cmrvqjvrn000alcsw216ijgbl", "stat</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>/api/draws/winners/cmrvqk5vb0049lcsg5y5vtfki</t>
+          <t>/api/draws/winners/cmrvqsfx6004slcsg3uve7y2u</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -1291,7 +1291,7 @@
         <v>200</v>
       </c>
       <c r="L14" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>

</xml_diff>